<commit_message>
Ajusta campos do ativo, adiciona responsável no form e campos técnicos dinâmicos e atualiza importador
</commit_message>
<xml_diff>
--- a/public/planilha_exemplo.xlsx
+++ b/public/planilha_exemplo.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:M4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -428,6 +428,15 @@
         <v>Situação</v>
       </c>
       <c r="J1" t="str">
+        <v>Processador</v>
+      </c>
+      <c r="K1" t="str">
+        <v>Sistema Operacional</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Nome da máquina</v>
+      </c>
+      <c r="M1" t="str">
         <v>OBS</v>
       </c>
     </row>
@@ -460,6 +469,15 @@
         <v>Boa</v>
       </c>
       <c r="J2" t="str">
+        <v>Ryzen 5</v>
+      </c>
+      <c r="K2" t="str">
+        <v>Windows 11</v>
+      </c>
+      <c r="L2" t="str">
+        <v>NTB-DANIELE</v>
+      </c>
+      <c r="M2" t="str">
         <v>Sem observações</v>
       </c>
     </row>
@@ -492,6 +510,15 @@
         <v>Boa</v>
       </c>
       <c r="J3" t="str">
+        <v>Core i7</v>
+      </c>
+      <c r="K3" t="str">
+        <v>Ubuntu 22.04</v>
+      </c>
+      <c r="L3" t="str">
+        <v>SRV-FELIPE</v>
+      </c>
+      <c r="M3" t="str">
         <v>Teclado trocado</v>
       </c>
     </row>
@@ -524,12 +551,21 @@
         <v>Critico</v>
       </c>
       <c r="J4" t="str">
+        <v>Core i5</v>
+      </c>
+      <c r="K4" t="str">
+        <v>Windows 10</v>
+      </c>
+      <c r="L4" t="str">
+        <v>NTB-ADRIANA</v>
+      </c>
+      <c r="M4" t="str">
         <v>Diversos travamentos, máquina descontinuada</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
reestruturação da aba de ativos
</commit_message>
<xml_diff>
--- a/public/planilha_exemplo.xlsx
+++ b/public/planilha_exemplo.xlsx
@@ -3,8 +3,13 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Ativos" sheetId="1" r:id="rId1"/>
+    <sheet name="Importação de ativos" sheetId="1" r:id="rId1"/>
+    <sheet name="Instruções" sheetId="2" r:id="rId2"/>
+    <sheet name="Valores permitidos" sheetId="3" r:id="rId3"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Importação de ativos'!A1:Y5</definedName>
+  </definedNames>
 </workbook>
 </file>
 
@@ -397,175 +402,590 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M4"/>
+  <dimension ref="A1:Y5"/>
+  <cols>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="21.83203125" customWidth="1"/>
+    <col min="3" max="3" width="13.83203125" customWidth="1"/>
+    <col min="4" max="4" width="15.83203125" customWidth="1"/>
+    <col min="5" max="5" width="23.83203125" customWidth="1"/>
+    <col min="6" max="6" width="21.83203125" customWidth="1"/>
+    <col min="7" max="7" width="23.83203125" customWidth="1"/>
+    <col min="8" max="8" width="11.83203125" customWidth="1"/>
+    <col min="9" max="9" width="16.83203125" customWidth="1"/>
+    <col min="10" max="10" width="11.83203125" customWidth="1"/>
+    <col min="11" max="11" width="41.83203125" customWidth="1"/>
+    <col min="12" max="12" width="22.83203125" customWidth="1"/>
+    <col min="13" max="13" width="22.83203125" customWidth="1"/>
+    <col min="14" max="14" width="14.83203125" customWidth="1"/>
+    <col min="15" max="15" width="14.83203125" customWidth="1"/>
+    <col min="16" max="16" width="16.83203125" customWidth="1"/>
+    <col min="17" max="17" width="22.83203125" customWidth="1"/>
+    <col min="18" max="18" width="20.83203125" customWidth="1"/>
+    <col min="19" max="19" width="16.83203125" customWidth="1"/>
+    <col min="20" max="20" width="32.83203125" customWidth="1"/>
+    <col min="21" max="21" width="20.83203125" customWidth="1"/>
+    <col min="22" max="22" width="21.83203125" customWidth="1"/>
+    <col min="23" max="23" width="14.83203125" customWidth="1"/>
+    <col min="24" max="24" width="15.83203125" customWidth="1"/>
+    <col min="25" max="25" width="14.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>User</v>
+        <v>categoria_ativo</v>
       </c>
       <c r="B1" t="str">
-        <v>Setor</v>
+        <v>nome_maquina</v>
       </c>
       <c r="C1" t="str">
-        <v>Equipamento</v>
+        <v>patrimonio</v>
       </c>
       <c r="D1" t="str">
-        <v>Modelo</v>
+        <v>numero_serie</v>
       </c>
       <c r="E1" t="str">
-        <v>Patrimonio</v>
+        <v>numero_serie_teclado</v>
       </c>
       <c r="F1" t="str">
-        <v>Coligada</v>
+        <v>numero_serie_mouse</v>
       </c>
       <c r="G1" t="str">
-        <v>Numero de Serie</v>
+        <v>numero_serie_headset</v>
       </c>
       <c r="H1" t="str">
-        <v>Ano</v>
+        <v>marca</v>
       </c>
       <c r="I1" t="str">
-        <v>Situação</v>
+        <v>modelo</v>
       </c>
       <c r="J1" t="str">
-        <v>Processador</v>
+        <v>condicao</v>
       </c>
       <c r="K1" t="str">
-        <v>Sistema Operacional</v>
+        <v>observacoes</v>
       </c>
       <c r="L1" t="str">
-        <v>Nome da máquina</v>
+        <v>usuario_responsavel</v>
       </c>
       <c r="M1" t="str">
-        <v>OBS</v>
+        <v>email_usuario</v>
+      </c>
+      <c r="N1" t="str">
+        <v>ano_produto</v>
+      </c>
+      <c r="O1" t="str">
+        <v>localizacao</v>
+      </c>
+      <c r="P1" t="str">
+        <v>processador</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>sistema_operacional</v>
+      </c>
+      <c r="R1" t="str">
+        <v>endereco_mac</v>
+      </c>
+      <c r="S1" t="str">
+        <v>endereco_ip</v>
+      </c>
+      <c r="T1" t="str">
+        <v>chave_licenca_windows</v>
+      </c>
+      <c r="U1" t="str">
+        <v>tamanho_polegadas</v>
+      </c>
+      <c r="V1" t="str">
+        <v>numero_nota_fiscal</v>
+      </c>
+      <c r="W1" t="str">
+        <v>data_compra</v>
+      </c>
+      <c r="X1" t="str">
+        <v>valor_compra</v>
+      </c>
+      <c r="Y1" t="str">
+        <v>fornecedor</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
+        <v>Notebook</v>
+      </c>
+      <c r="B2" t="str">
+        <v>NOTE-FINANCEIRO-01</v>
+      </c>
+      <c r="C2" t="str">
+        <v>PAT-0001</v>
+      </c>
+      <c r="D2" t="str">
+        <v>SN123456</v>
+      </c>
+      <c r="E2" t="str">
+        <v/>
+      </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
+      <c r="H2" t="str">
+        <v>Dell</v>
+      </c>
+      <c r="I2" t="str">
+        <v>Latitude 5440</v>
+      </c>
+      <c r="J2" t="str">
+        <v>Boa</v>
+      </c>
+      <c r="K2" t="str">
+        <v>Exemplo de preenchimento para notebook</v>
+      </c>
+      <c r="L2" t="str">
         <v>Daniele Gomes</v>
       </c>
-      <c r="B2" t="str">
-        <v>Financeiro</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Notebook</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Dell Vostro 15 3525</v>
-      </c>
-      <c r="E2" t="str">
-        <v>000024</v>
-      </c>
-      <c r="F2" t="str">
-        <v>UNIQO</v>
-      </c>
-      <c r="G2" t="str">
-        <v>67CB7X3</v>
-      </c>
-      <c r="H2" t="str">
-        <v>2023</v>
-      </c>
-      <c r="I2" t="str">
-        <v>Boa</v>
-      </c>
-      <c r="J2" t="str">
-        <v>Ryzen 5</v>
-      </c>
-      <c r="K2" t="str">
-        <v>Windows 11</v>
-      </c>
-      <c r="L2" t="str">
-        <v>NTB-DANIELE</v>
-      </c>
       <c r="M2" t="str">
-        <v>Sem observações</v>
+        <v>daniele@empresa.com</v>
+      </c>
+      <c r="N2" t="str">
+        <v>2025</v>
+      </c>
+      <c r="O2" t="str">
+        <v>Sede RJ</v>
+      </c>
+      <c r="P2" t="str">
+        <v>Intel Core i5</v>
+      </c>
+      <c r="Q2" t="str">
+        <v>Windows 11 Pro</v>
+      </c>
+      <c r="R2" t="str">
+        <v>00:1A:2B:3C:4D:5E</v>
+      </c>
+      <c r="S2" t="str">
+        <v>192.168.1.100</v>
+      </c>
+      <c r="T2" t="str">
+        <v>XXXXX-XXXXX-XXXXX-XXXXX-XXXXX</v>
+      </c>
+      <c r="U2" t="str">
+        <v/>
+      </c>
+      <c r="V2" t="str">
+        <v>NF-9988</v>
+      </c>
+      <c r="W2" t="str">
+        <v>2025-01-10</v>
+      </c>
+      <c r="X2" t="str">
+        <v>4500.00</v>
+      </c>
+      <c r="Y2" t="str">
+        <v>Dell Brasil</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
+        <v>Monitor</v>
+      </c>
+      <c r="B3" t="str">
+        <v/>
+      </c>
+      <c r="C3" t="str">
+        <v>PAT-0002</v>
+      </c>
+      <c r="D3" t="str">
+        <v>MON123456</v>
+      </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+      <c r="G3" t="str">
+        <v/>
+      </c>
+      <c r="H3" t="str">
+        <v>LG</v>
+      </c>
+      <c r="I3" t="str">
+        <v>24MP400</v>
+      </c>
+      <c r="J3" t="str">
+        <v>Boa</v>
+      </c>
+      <c r="K3" t="str">
+        <v>Exemplo de monitor</v>
+      </c>
+      <c r="L3" t="str">
         <v>Felipe Silva</v>
       </c>
-      <c r="B3" t="str">
-        <v>T.I</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Notebook</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Dell Vostro 14 5490</v>
-      </c>
-      <c r="E3" t="str">
-        <v>000080</v>
-      </c>
-      <c r="F3" t="str">
-        <v>VIVERDE</v>
-      </c>
-      <c r="G3" t="str">
-        <v>2C3CH73</v>
-      </c>
-      <c r="H3" t="str">
-        <v>2020</v>
-      </c>
-      <c r="I3" t="str">
-        <v>Boa</v>
-      </c>
-      <c r="J3" t="str">
-        <v>Core i7</v>
-      </c>
-      <c r="K3" t="str">
-        <v>Ubuntu 22.04</v>
-      </c>
-      <c r="L3" t="str">
-        <v>SRV-FELIPE</v>
-      </c>
       <c r="M3" t="str">
-        <v>Teclado trocado</v>
+        <v>felipe@empresa.com</v>
+      </c>
+      <c r="N3" t="str">
+        <v/>
+      </c>
+      <c r="O3" t="str">
+        <v>Sede RJ</v>
+      </c>
+      <c r="P3" t="str">
+        <v/>
+      </c>
+      <c r="Q3" t="str">
+        <v/>
+      </c>
+      <c r="R3" t="str">
+        <v/>
+      </c>
+      <c r="S3" t="str">
+        <v/>
+      </c>
+      <c r="T3" t="str">
+        <v/>
+      </c>
+      <c r="U3" t="str">
+        <v>24</v>
+      </c>
+      <c r="V3" t="str">
+        <v>NF-5544</v>
+      </c>
+      <c r="W3" t="str">
+        <v>2024-05-15</v>
+      </c>
+      <c r="X3" t="str">
+        <v>890.00</v>
+      </c>
+      <c r="Y3" t="str">
+        <v>Kabum</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
+        <v>Kit teclado e mouse</v>
+      </c>
+      <c r="B4" t="str">
+        <v/>
+      </c>
+      <c r="C4" t="str">
+        <v>PAT-0003</v>
+      </c>
+      <c r="D4" t="str">
+        <v/>
+      </c>
+      <c r="E4" t="str">
+        <v>TEC123456</v>
+      </c>
+      <c r="F4" t="str">
+        <v>MOU123456</v>
+      </c>
+      <c r="G4" t="str">
+        <v/>
+      </c>
+      <c r="H4" t="str">
+        <v>Logitech</v>
+      </c>
+      <c r="I4" t="str">
+        <v>MK540</v>
+      </c>
+      <c r="J4" t="str">
+        <v>Boa</v>
+      </c>
+      <c r="K4" t="str">
+        <v>Exemplo de Kit Teclado e Mouse</v>
+      </c>
+      <c r="L4" t="str">
         <v>Adriana Moura</v>
       </c>
+      <c r="M4" t="str">
+        <v>adriana@empresa.com</v>
+      </c>
+      <c r="N4" t="str">
+        <v/>
+      </c>
+      <c r="O4" t="str">
+        <v>Sede RJ</v>
+      </c>
+      <c r="P4" t="str">
+        <v/>
+      </c>
+      <c r="Q4" t="str">
+        <v/>
+      </c>
+      <c r="R4" t="str">
+        <v/>
+      </c>
+      <c r="S4" t="str">
+        <v/>
+      </c>
+      <c r="T4" t="str">
+        <v/>
+      </c>
+      <c r="U4" t="str">
+        <v/>
+      </c>
+      <c r="V4" t="str">
+        <v/>
+      </c>
+      <c r="W4" t="str">
+        <v/>
+      </c>
+      <c r="X4" t="str">
+        <v/>
+      </c>
+      <c r="Y4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Headset</v>
+      </c>
+      <c r="B5" t="str">
+        <v/>
+      </c>
+      <c r="C5" t="str">
+        <v>PAT-0004</v>
+      </c>
+      <c r="D5" t="str">
+        <v/>
+      </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+      <c r="G5" t="str">
+        <v>HEAD123456</v>
+      </c>
+      <c r="H5" t="str">
+        <v>Jabra</v>
+      </c>
+      <c r="I5" t="str">
+        <v>Evolve 20</v>
+      </c>
+      <c r="J5" t="str">
+        <v>Boa</v>
+      </c>
+      <c r="K5" t="str">
+        <v>Exemplo de Headset</v>
+      </c>
+      <c r="L5" t="str">
+        <v>Daniele Gomes</v>
+      </c>
+      <c r="M5" t="str">
+        <v>daniele@empresa.com</v>
+      </c>
+      <c r="N5" t="str">
+        <v/>
+      </c>
+      <c r="O5" t="str">
+        <v>Sede RJ</v>
+      </c>
+      <c r="P5" t="str">
+        <v/>
+      </c>
+      <c r="Q5" t="str">
+        <v/>
+      </c>
+      <c r="R5" t="str">
+        <v/>
+      </c>
+      <c r="S5" t="str">
+        <v/>
+      </c>
+      <c r="T5" t="str">
+        <v/>
+      </c>
+      <c r="U5" t="str">
+        <v/>
+      </c>
+      <c r="V5" t="str">
+        <v/>
+      </c>
+      <c r="W5" t="str">
+        <v/>
+      </c>
+      <c r="X5" t="str">
+        <v/>
+      </c>
+      <c r="Y5" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:Y5"/>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:Y5"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B12"/>
+  <cols>
+    <col min="1" max="1" width="30.83203125" customWidth="1"/>
+    <col min="2" max="2" width="90.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Instrução</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Detalhes</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>1. Categorias aceitas</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Notebook, Monitor, Kit teclado e mouse, Headset (Case-insensitive).</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>2. Notebook - Obrigatórios</v>
+      </c>
+      <c r="B3" t="str">
+        <v>nome_maquina, numero_serie, patrimonio, marca, modelo, condicao, localizacao.</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>3. Monitor - Obrigatórios</v>
+      </c>
       <c r="B4" t="str">
-        <v>Juridico</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Notebook</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Dell Vostro 5490</v>
-      </c>
-      <c r="E4" t="str">
-        <v>000010</v>
-      </c>
-      <c r="F4" t="str">
-        <v>DA</v>
-      </c>
-      <c r="G4" t="str">
-        <v>BDYKD53</v>
-      </c>
-      <c r="H4" t="str">
-        <v>2020</v>
-      </c>
-      <c r="I4" t="str">
-        <v>Critico</v>
-      </c>
-      <c r="J4" t="str">
-        <v>Core i5</v>
-      </c>
-      <c r="K4" t="str">
-        <v>Windows 10</v>
-      </c>
-      <c r="L4" t="str">
-        <v>NTB-ADRIANA</v>
-      </c>
-      <c r="M4" t="str">
-        <v>Diversos travamentos, máquina descontinuada</v>
+        <v>patrimonio, numero_serie, marca, modelo, tamanho_polegadas, condicao, localizacao.</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>4. Kit teclado e mouse - Obrigatórios</v>
+      </c>
+      <c r="B5" t="str">
+        <v>numero_serie_teclado, numero_serie_mouse, marca, modelo, condicao, localizacao.</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>5. Headset - Obrigatórios</v>
+      </c>
+      <c r="B6" t="str">
+        <v>numero_serie_headset, marca, modelo, condicao, localizacao.</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>6. Condições aceitas</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Boa, Média, Ruim (ou 'Media').</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>7. Formato MAC</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Exemplo: 00:1A:2B:3C:4D:5E.</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>8. Formato IP</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Exemplo: 192.168.1.100.</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>9. Ano do produto</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Número de 4 dígitos entre 1900 e 2100 (ex: 2025).</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>10. Usuário Responsável</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Preencha com o nome ou e-mail exato do colaborador cadastrado.</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>11. Localização</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Preencha com o nome exato da localização cadastrada.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B12"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:B5"/>
+  <cols>
+    <col min="1" max="1" width="30.83203125" customWidth="1"/>
+    <col min="2" max="2" width="30.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>Categorias Disponíveis</v>
+      </c>
+      <c r="B1" t="str">
+        <v>Condições Aceitas</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Notebook</v>
+      </c>
+      <c r="B2" t="str">
+        <v>Boa</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Monitor</v>
+      </c>
+      <c r="B3" t="str">
+        <v>Média</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Kit teclado e mouse</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Ruim</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Headset</v>
+      </c>
+      <c r="B5" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:B5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>